<commit_message>
current resistors are added to variants; rooms are rearranged
</commit_message>
<xml_diff>
--- a/Project Outputs for c1-12/ChipSet.xlsx
+++ b/Project Outputs for c1-12/ChipSet.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr/>
+  <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\D\Proj\DistrHall\git\Hall_module_board\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Your files\Volkovao\projects_ovolkova2\Hall_module_board\Project Outputs for c1-12\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14376" windowHeight="10212"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14370" windowHeight="10215"/>
   </bookViews>
   <sheets>
     <sheet name="PCB_proj_module_1_1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="152511" refMode="R1C1"/>
+  <calcPr calcId="162913" refMode="R1C1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -816,7 +816,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;₽&quot;"/>
     <numFmt numFmtId="165" formatCode="#,##0\ &quot;₽&quot;"/>
@@ -1283,19 +1283,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H83"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="29.21875" customWidth="1"/>
+    <col min="1" max="1" width="29.28515625" customWidth="1"/>
     <col min="2" max="2" width="44" customWidth="1"/>
-    <col min="3" max="3" width="40.33203125" customWidth="1"/>
-    <col min="4" max="4" width="100.21875" customWidth="1"/>
-    <col min="5" max="5" width="13.6640625" customWidth="1"/>
-    <col min="6" max="6" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.33203125" customWidth="1"/>
-    <col min="8" max="8" width="61.44140625" customWidth="1"/>
+    <col min="3" max="3" width="40.28515625" customWidth="1"/>
+    <col min="4" max="4" width="100.28515625" customWidth="1"/>
+    <col min="5" max="5" width="13.7109375" customWidth="1"/>
+    <col min="6" max="6" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.28515625" customWidth="1"/>
+    <col min="8" max="8" width="61.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1315,7 +1315,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -1335,7 +1335,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="18" t="s">
         <v>130</v>
       </c>
@@ -1362,7 +1362,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="21" t="s">
         <v>187</v>
       </c>
@@ -1373,7 +1373,7 @@
       <c r="F4" s="5"/>
       <c r="G4" s="5"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>68</v>
       </c>
@@ -1397,7 +1397,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>66</v>
       </c>
@@ -1421,7 +1421,7 @@
         <v>5960</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>96</v>
       </c>
@@ -1445,7 +1445,7 @@
         <v>22400</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>94</v>
       </c>
@@ -1469,7 +1469,7 @@
         <v>11120</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>111</v>
       </c>
@@ -1493,7 +1493,7 @@
         <v>940</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>83</v>
       </c>
@@ -1517,7 +1517,7 @@
         <v>510</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>71</v>
       </c>
@@ -1541,7 +1541,7 @@
         <v>1570</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>87</v>
       </c>
@@ -1565,7 +1565,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>90</v>
       </c>
@@ -1589,7 +1589,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>27</v>
       </c>
@@ -1613,7 +1613,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>92</v>
       </c>
@@ -1637,7 +1637,7 @@
         <v>1460</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>79</v>
       </c>
@@ -1661,7 +1661,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>81</v>
       </c>
@@ -1685,7 +1685,7 @@
         <v>12800</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>98</v>
       </c>
@@ -1709,7 +1709,7 @@
         <v>16800</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>215</v>
       </c>
@@ -1733,7 +1733,7 @@
         <v>2710</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>85</v>
       </c>
@@ -1757,7 +1757,7 @@
         <v>3800</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>75</v>
       </c>
@@ -1781,7 +1781,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>73</v>
       </c>
@@ -1803,7 +1803,7 @@
         <v>4850</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="20"/>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
@@ -1812,7 +1812,7 @@
       <c r="F23" s="5"/>
       <c r="G23" s="5"/>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="21" t="s">
         <v>186</v>
       </c>
@@ -1823,7 +1823,7 @@
       <c r="F24" s="5"/>
       <c r="G24" s="5"/>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>145</v>
       </c>
@@ -1847,7 +1847,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="8" t="s">
         <v>168</v>
       </c>
@@ -1869,7 +1869,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>140</v>
       </c>
@@ -1893,7 +1893,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="8" t="s">
         <v>162</v>
       </c>
@@ -1920,7 +1920,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="8" t="s">
         <v>165</v>
       </c>
@@ -1942,7 +1942,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="8" t="s">
         <v>170</v>
       </c>
@@ -1964,7 +1964,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>126</v>
       </c>
@@ -1988,7 +1988,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="21"/>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
@@ -1997,7 +1997,7 @@
       <c r="F32" s="5"/>
       <c r="G32" s="5"/>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="21" t="s">
         <v>182</v>
       </c>
@@ -2008,7 +2008,7 @@
       <c r="F33" s="5"/>
       <c r="G33" s="5"/>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>175</v>
       </c>
@@ -2032,7 +2032,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>44</v>
       </c>
@@ -2056,7 +2056,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>46</v>
       </c>
@@ -2080,7 +2080,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="37" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>181</v>
       </c>
@@ -2107,7 +2107,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="8" t="s">
         <v>147</v>
       </c>
@@ -2134,7 +2134,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>143</v>
       </c>
@@ -2158,7 +2158,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>138</v>
       </c>
@@ -2185,7 +2185,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" s="8" t="s">
         <v>157</v>
       </c>
@@ -2209,7 +2209,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="8"/>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
@@ -2218,7 +2218,7 @@
       <c r="F42" s="5"/>
       <c r="G42" s="5"/>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="20" t="s">
         <v>188</v>
       </c>
@@ -2229,7 +2229,7 @@
       <c r="F43" s="5"/>
       <c r="G43" s="5"/>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>20</v>
       </c>
@@ -2253,7 +2253,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>22</v>
       </c>
@@ -2277,7 +2277,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>24</v>
       </c>
@@ -2300,7 +2300,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>15</v>
       </c>
@@ -2324,7 +2324,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>77</v>
       </c>
@@ -2348,7 +2348,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" s="17" t="s">
         <v>128</v>
       </c>
@@ -2372,7 +2372,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" s="17"/>
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
@@ -2381,7 +2381,7 @@
       <c r="F50" s="5"/>
       <c r="G50" s="5"/>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" s="22" t="s">
         <v>197</v>
       </c>
@@ -2392,7 +2392,7 @@
       <c r="F51" s="5"/>
       <c r="G51" s="5"/>
     </row>
-    <row r="52" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="9" t="s">
         <v>35</v>
       </c>
@@ -2417,7 +2417,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>38</v>
       </c>
@@ -2441,7 +2441,7 @@
         <v>780</v>
       </c>
     </row>
-    <row r="54" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="9" t="s">
         <v>112</v>
       </c>
@@ -2468,7 +2468,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" s="22"/>
       <c r="B55" s="2"/>
       <c r="C55" s="2"/>
@@ -2477,7 +2477,7 @@
       <c r="F55" s="5"/>
       <c r="G55" s="5"/>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" s="22" t="s">
         <v>189</v>
       </c>
@@ -2488,7 +2488,7 @@
       <c r="F56" s="5"/>
       <c r="G56" s="5"/>
     </row>
-    <row r="57" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>113</v>
       </c>
@@ -2512,7 +2512,7 @@
         <v>313.60000000000002</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" s="8" t="s">
         <v>114</v>
       </c>
@@ -2536,7 +2536,7 @@
         <v>83.6</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
         <v>117</v>
       </c>
@@ -2560,7 +2560,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="60" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="9" t="s">
         <v>8</v>
       </c>
@@ -2583,7 +2583,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="61" spans="1:8" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:8" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="13" t="s">
         <v>8</v>
       </c>
@@ -2606,7 +2606,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="62" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="13"/>
       <c r="B62" s="13"/>
       <c r="C62" s="13"/>
@@ -2615,7 +2615,7 @@
       <c r="F62" s="16"/>
       <c r="G62" s="16"/>
     </row>
-    <row r="63" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="23" t="s">
         <v>190</v>
       </c>
@@ -2626,7 +2626,7 @@
       <c r="F63" s="16"/>
       <c r="G63" s="16"/>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
         <v>60</v>
       </c>
@@ -2648,7 +2648,7 @@
         <v>2800</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" s="8" t="s">
         <v>226</v>
       </c>
@@ -2675,7 +2675,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
         <v>220</v>
       </c>
@@ -2702,7 +2702,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
         <v>225</v>
       </c>
@@ -2729,7 +2729,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
         <v>228</v>
       </c>
@@ -2756,7 +2756,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
         <v>48</v>
       </c>
@@ -2778,7 +2778,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
         <v>50</v>
       </c>
@@ -2800,7 +2800,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
         <v>52</v>
       </c>
@@ -2822,7 +2822,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
         <v>54</v>
       </c>
@@ -2844,7 +2844,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
         <v>56</v>
       </c>
@@ -2866,7 +2866,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
         <v>58</v>
       </c>
@@ -2888,7 +2888,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75" s="23" t="s">
         <v>196</v>
       </c>
@@ -2899,7 +2899,7 @@
       <c r="F75" s="5"/>
       <c r="G75" s="5"/>
     </row>
-    <row r="76" spans="1:8" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:8" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
         <v>194</v>
       </c>
@@ -2923,7 +2923,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
         <v>202</v>
       </c>
@@ -2947,7 +2947,7 @@
         <v>7140</v>
       </c>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
         <v>63</v>
       </c>
@@ -2971,7 +2971,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
         <v>100</v>
       </c>
@@ -2993,7 +2993,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
         <v>103</v>
       </c>
@@ -3013,7 +3013,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
         <v>235</v>
       </c>
@@ -3035,7 +3035,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
         <v>107</v>
       </c>
@@ -3057,7 +3057,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F83" s="5"/>
       <c r="G83" s="7">
         <f>SUM(G2:G82)</f>

</xml_diff>